<commit_message>
Label bill-checkup lever tiers, scope session cookie via COOKIE_DOMAIN, route provider.whollar.ca
- bill-checkup: heading above each lever tier (yours / Whollar / agreement)
- cookies.js: Domain attribute from COOKIE_DOMAIN (localhost = host-only) so
  www and provider subdomains share one session
- vercel.json: host-based rewrites for provider.whollar.ca / and /login
- pricing sheet update + 50-bill checkup test results

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PlanSavvy-Pricing.xlsx
+++ b/PlanSavvy-Pricing.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cell Phone Plans" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internet Plans" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TV Plans" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Plans" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cell Phone Plans" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Internet Plans" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TV Plans" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="All Plans" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'All Plans'!$A$1:$H$443</definedName>
@@ -7405,21 +7405,21 @@
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>EBOX</t>
+          <t>Bell</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>FTTN 50</t>
+          <t>Fibe 1.5 Gig (w/ Rogers or Fido mobile)</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>50 Mbps</t>
+          <t>1500 Mbps</t>
         </is>
       </c>
       <c r="F64" s="6" t="n">
-        <v>49.95</v>
+        <v>55</v>
       </c>
       <c r="G64" s="6" t="n"/>
     </row>

</xml_diff>